<commit_message>
feat: update brand colors and enhance Excel output formatting
</commit_message>
<xml_diff>
--- a/test_output.xlsx
+++ b/test_output.xlsx
@@ -11,7 +11,11 @@
     <sheet name="Line Items" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Automation Report" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Invoice Summary'!$A$1:$H$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Line Items'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Automation Report'!$A$1:$C$22</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -23,7 +27,7 @@
     <numFmt numFmtId="165" formatCode="mmm dd, yyyy"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,14 +38,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="16"/>
+      <color rgb="001F3A5F"/>
+      <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="18"/>
+      <sz val="26"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -51,7 +55,7 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="001F3A5F"/>
       <sz val="10"/>
     </font>
     <font>
@@ -63,23 +67,25 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001A1F2B"/>
+      <color rgb="001A1A1A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A1A1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B7791F"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00555555"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -99,26 +105,44 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="001F3A5F"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00888888"/>
+      <color rgb="00666666"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -148,12 +172,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="001F3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
+        <fgColor rgb="00EAF3FB"/>
       </patternFill>
     </fill>
     <fill>
@@ -163,11 +187,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F7FC"/>
+        <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -176,140 +200,212 @@
       <diagonal/>
     </border>
     <border>
+      <bottom style="thin">
+        <color rgb="002E75B6"/>
+      </bottom>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00C9D6E6"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00C9D6E6"/>
+      </right>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9D6E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9D6E6"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="001F3A5F"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9D6E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9D6E6"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00C9D6E6"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9D6E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9D6E6"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00C9D6E6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9D6E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9D6E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D6E6"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00C9D6E6"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="001F3A5F"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="11" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="11" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -675,23 +771,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1"/>
-    <row r="2" ht="26" customHeight="1">
+    <row r="2" ht="32" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>[Your Company Name]</t>
@@ -703,7 +799,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1">
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>[Street Address  ·  City, State ZIP  ·  (000) 000-0000  ·  email@domain.com]</t>
@@ -741,281 +837,281 @@
           <t>Acme Buyer LLC</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="10" t="n">
         <v>46169</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>123 Buyer St</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="10" t="n">
         <v>46199</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Springfield, IL 62704</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>✓ Paid / Unpaid</t>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>UNPAID</t>
         </is>
       </c>
     </row>
     <row r="11"/>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F12" s="15" t="inlineStr">
         <is>
           <t>Tax %</t>
         </is>
       </c>
-      <c r="G12" s="11" t="inlineStr">
+      <c r="G12" s="15" t="inlineStr">
         <is>
           <t>Tax Amt</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="15" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="12" t="n">
+      <c r="A13" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Office Furniture Set (Executive)</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>Northwind Trading Co.</t>
         </is>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="18" t="n">
         <v>1250</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="20">
         <f>D13*E13*F13</f>
         <v/>
       </c>
-      <c r="H13" s="17">
+      <c r="H13" s="21">
         <f>D13*E13+G13</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="18" t="n">
+      <c r="A14" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>Ergonomic Office Chairs</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>Northwind Trading Co.</t>
         </is>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="24" t="n">
         <v>185</v>
       </c>
-      <c r="F14" s="21" t="n">
+      <c r="F14" s="25" t="n">
         <v>0.18</v>
       </c>
-      <c r="G14" s="22">
+      <c r="G14" s="26">
         <f>D14*E14*F14</f>
         <v/>
       </c>
-      <c r="H14" s="23">
+      <c r="H14" s="27">
         <f>D14*E14+G14</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="12" t="n">
+      <c r="A15" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Conference Room Table</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>Northwind Trading Co.</t>
         </is>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="18" t="n">
         <v>890</v>
       </c>
-      <c r="F15" s="15" t="n">
+      <c r="F15" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="20">
         <f>D15*E15*F15</f>
         <v/>
       </c>
-      <c r="H15" s="17">
+      <c r="H15" s="21">
         <f>D15*E15+G15</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="18" t="n">
+      <c r="A16" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>Storage Cabinets (4-drawer)</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C16" s="23" t="inlineStr">
         <is>
           <t>Northwind Trading Co.</t>
         </is>
       </c>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="24" t="n">
         <v>220</v>
       </c>
-      <c r="F16" s="21" t="n">
+      <c r="F16" s="25" t="n">
         <v>0.18</v>
       </c>
-      <c r="G16" s="22">
+      <c r="G16" s="26">
         <f>D16*E16*F16</f>
         <v/>
       </c>
-      <c r="H16" s="23">
+      <c r="H16" s="27">
         <f>D16*E16+G16</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Installation &amp; Setup Service</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>Northwind Trading Co.</t>
         </is>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="E17" s="18" t="n">
         <v>350</v>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="F17" s="19" t="n">
         <v>0.18</v>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="20">
         <f>D17*E17*F17</f>
         <v/>
       </c>
-      <c r="H17" s="17">
+      <c r="H17" s="21">
         <f>D17*E17+G17</f>
         <v/>
       </c>
     </row>
     <row r="18"/>
     <row r="19" ht="18" customHeight="1">
-      <c r="F19" s="24" t="inlineStr">
+      <c r="F19" s="28" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="H19" s="25">
+      <c r="H19" s="29">
         <f>SUMPRODUCT(D13:D17,E13:E17)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="F20" s="24" t="inlineStr">
+      <c r="F20" s="28" t="inlineStr">
         <is>
           <t>Tax</t>
         </is>
       </c>
-      <c r="H20" s="25">
+      <c r="H20" s="29">
         <f>SUM(G13:G17)</f>
         <v/>
       </c>
     </row>
     <row r="21"/>
     <row r="22" ht="26" customHeight="1">
-      <c r="E22" s="26" t="inlineStr">
+      <c r="E22" s="30" t="inlineStr">
         <is>
           <t>TOTAL DUE</t>
         </is>
       </c>
-      <c r="H22" s="27">
+      <c r="H22" s="31">
         <f>SUM(H13:H17)</f>
         <v/>
       </c>
@@ -1023,28 +1119,28 @@
     <row r="23"/>
     <row r="24"/>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="32" t="inlineStr">
         <is>
           <t>Payment Terms</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="33" t="inlineStr">
         <is>
           <t>Payment due within 30 days of invoice date.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="33" t="inlineStr">
         <is>
           <t>Bank transfer preferred  ·  [Bank Name · Account # · Routing #]</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="33" t="inlineStr">
         <is>
           <t>Questions?  [your@email.com]</t>
         </is>
@@ -1052,40 +1148,59 @@
     </row>
     <row r="29"/>
     <row r="30"/>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="29" t="inlineStr">
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="34" t="inlineStr">
         <is>
           <t>Thank you for your business.</t>
         </is>
       </c>
-      <c r="E31" s="30" t="inlineStr">
+    </row>
+    <row r="32"/>
+    <row r="33" ht="28" customHeight="1">
+      <c r="F33" s="35" t="inlineStr"/>
+    </row>
+    <row r="34" ht="14" customHeight="1">
+      <c r="F34" s="36" t="inlineStr">
+        <is>
+          <t>Authorized Signature</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="37" t="inlineStr">
         <is>
           <t>[Your Name]  ·  Finance Automation Specialist  ·  yourwebsite.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="E31:H31"/>
+  <mergeCells count="21">
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="E3:H3"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A3:D3"/>
     <mergeCell ref="G10:H10"/>
-    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="E22:G22"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A26:D26"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A31:H31"/>
     <mergeCell ref="E2:H2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1093,15 +1208,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -1109,12 +1224,12 @@
   <sheetData>
     <row r="1"/>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="31" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>Line Item Detail</t>
         </is>
       </c>
-      <c r="E2" s="32" t="inlineStr">
+      <c r="E2" s="39" t="inlineStr">
         <is>
           <t>INV-2026-0584  ·  Northwind Trading Co.</t>
         </is>
@@ -1122,239 +1237,257 @@
     </row>
     <row r="3"/>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Invoice #</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>sample_invoice.pdf</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>INV-2026-0584</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Office Furniture Set (Executive)</t>
         </is>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="18" t="n">
         <v>1250</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="18" t="n">
         <v>2500</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="18" t="n">
+      <c r="A6" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>sample_invoice.pdf</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>INV-2026-0584</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>Ergonomic Office Chairs</t>
         </is>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="24" t="n">
         <v>185</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G6" s="24" t="n">
         <v>1480</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="12" t="n">
+      <c r="A7" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>sample_invoice.pdf</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>INV-2026-0584</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Conference Room Table</t>
         </is>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="18" t="n">
         <v>890</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="18" t="n">
         <v>890</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="18" t="n">
+      <c r="A8" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>sample_invoice.pdf</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>INV-2026-0584</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>Storage Cabinets (4-drawer)</t>
         </is>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="24" t="n">
         <v>220</v>
       </c>
-      <c r="G8" s="20" t="n">
+      <c r="G8" s="24" t="n">
         <v>880</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>sample_invoice.pdf</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>INV-2026-0584</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Installation &amp; Setup Service</t>
         </is>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="18" t="n">
         <v>350</v>
       </c>
-      <c r="G9" s="14" t="n">
+      <c r="G9" s="18" t="n">
         <v>350</v>
       </c>
     </row>
     <row r="10"/>
     <row r="11" ht="18" customHeight="1">
-      <c r="F11" s="24" t="inlineStr">
+      <c r="F11" s="28" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="G11" s="25" t="n">
+      <c r="G11" s="29" t="n">
         <v>6100</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="F12" s="24" t="inlineStr">
+      <c r="F12" s="28" t="inlineStr">
         <is>
           <t>Tax (18%)</t>
         </is>
       </c>
-      <c r="G12" s="25" t="n">
+      <c r="G12" s="29" t="n">
         <v>1098</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="F13" s="26" t="inlineStr">
+      <c r="F13" s="30" t="inlineStr">
         <is>
           <t>TOTAL DUE</t>
         </is>
       </c>
-      <c r="G13" s="27" t="n">
+      <c r="G13" s="31" t="n">
         <v>7198</v>
       </c>
     </row>
     <row r="14"/>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="34" t="inlineStr">
         <is>
           <t>Thank you for your business.</t>
         </is>
       </c>
-      <c r="D15" s="30" t="inlineStr">
+    </row>
+    <row r="16"/>
+    <row r="17" ht="28" customHeight="1">
+      <c r="E17" s="35" t="inlineStr"/>
+    </row>
+    <row r="18" ht="14" customHeight="1">
+      <c r="E18" s="36" t="inlineStr">
+        <is>
+          <t>Authorized Signature</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t>[Your Name]  ·  Finance Automation Specialist  ·  yourwebsite.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A15:C15"/>
+  <mergeCells count="6">
     <mergeCell ref="E2:G2"/>
-    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1362,24 +1495,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1"/>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="31" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>Automation Processing Report</t>
         </is>
       </c>
-      <c r="B2" s="33" t="inlineStr">
+      <c r="B2" s="40" t="inlineStr">
         <is>
           <t>Generated: May 29, 2026</t>
         </is>
@@ -1387,136 +1520,136 @@
     </row>
     <row r="3"/>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="34" t="inlineStr">
+      <c r="A5" s="41" t="inlineStr">
         <is>
           <t>Invoices processed</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>1 invoice</t>
         </is>
       </c>
-      <c r="C5" s="35" t="inlineStr">
+      <c r="C5" s="42" t="inlineStr">
         <is>
           <t>✓ OK</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="43" t="inlineStr">
         <is>
           <t>Successful extractions</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>1 of 1  (100%)</t>
         </is>
       </c>
-      <c r="C6" s="37" t="inlineStr">
+      <c r="C6" s="44" t="inlineStr">
         <is>
           <t>✓ OK</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>Failed / flagged</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C7" s="38" t="inlineStr">
+      <c r="C7" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="43" t="inlineStr">
         <is>
           <t>Total value captured</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>$7,198.00</t>
         </is>
       </c>
-      <c r="C8" s="37" t="inlineStr">
+      <c r="C8" s="44" t="inlineStr">
         <is>
           <t>✓ OK</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="34" t="inlineStr">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>Tax captured</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>$1,098.00</t>
         </is>
       </c>
-      <c r="C9" s="35" t="inlineStr">
+      <c r="C9" s="42" t="inlineStr">
         <is>
           <t>✓ OK</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="A10" s="43" t="inlineStr">
         <is>
           <t>Processing time</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>&lt; 4 seconds</t>
         </is>
       </c>
-      <c r="C10" s="37" t="inlineStr">
+      <c r="C10" s="44" t="inlineStr">
         <is>
           <t>✓ Fast</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="34" t="inlineStr">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>Manual entry required</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>0 fields</t>
         </is>
       </c>
-      <c r="C11" s="35" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>✓ None</t>
         </is>
@@ -1525,12 +1658,12 @@
     <row r="12"/>
     <row r="13"/>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>Want this running automatically for your business?</t>
         </is>
       </c>
-      <c r="B14" s="39" t="inlineStr">
+      <c r="B14" s="46" t="inlineStr">
         <is>
           <t>Book a free 30-min audit → yourwebsite.com</t>
         </is>
@@ -1538,24 +1671,43 @@
     </row>
     <row r="15"/>
     <row r="16"/>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="29" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="34" t="inlineStr">
         <is>
           <t>Thank you for your business.</t>
         </is>
       </c>
-      <c r="B17" s="30" t="inlineStr">
+    </row>
+    <row r="18"/>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="35" t="inlineStr"/>
+    </row>
+    <row r="20" ht="14" customHeight="1">
+      <c r="A20" s="36" t="inlineStr">
+        <is>
+          <t>Authorized Signature</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="37" t="inlineStr">
         <is>
           <t>[Your Name]  ·  Finance Automation Specialist  ·  yourwebsite.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A17:C17"/>
     <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="A20:C20"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>